<commit_message>
Fix leading-zero normalisation; regenerate report pipeline
unit_matcher.py: normalize_unit() now strips leading zeros so WE06
and 6 both produce canonical key suffix WE6 — eliminates all fuzzy
fallbacks, lifting audit_report match rate from 8 exact+7 fuzzy to
15/15 exact.

Regenerated artifacts:
  - data/audit_report_normalized.csv: all 15 rows now exact-matched
  - data/CROSS_REFERENCE_REPORT.xlsx: correct self-payer exclusion
    (WE3 Bornholmerstr.80, WE9 Residenzstr.129), 13 rows compared

Report result: 0 Action Required, 4 Review, 9 Correct.

https://claude.ai/code/session_01UHumaZ1fAHVpVwJmGiGLez
</commit_message>
<xml_diff>
--- a/data/CROSS_REFERENCE_REPORT.xlsx
+++ b/data/CROSS_REFERENCE_REPORT.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,30 +436,40 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>wp_hausgeld</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>wp_ruecklage</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>wp_total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>actual_payment</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>delta_monthly</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>delta_annual</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>match_confidence</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
@@ -476,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,30 +507,40 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>wp_hausgeld</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>wp_ruecklage</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>wp_total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>actual_payment</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>delta_monthly</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>delta_annual</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>match_confidence</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
@@ -543,23 +563,29 @@
         </is>
       </c>
       <c r="D2" t="n">
+        <v>289</v>
+      </c>
+      <c r="E2" t="n">
+        <v>98</v>
+      </c>
+      <c r="F2" t="n">
         <v>387</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>395</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>8</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>96</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
@@ -582,23 +608,29 @@
         </is>
       </c>
       <c r="D3" t="n">
+        <v>330</v>
+      </c>
+      <c r="E3" t="n">
+        <v>110</v>
+      </c>
+      <c r="F3" t="n">
         <v>440</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>445</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>60</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
@@ -621,23 +653,29 @@
         </is>
       </c>
       <c r="D4" t="n">
+        <v>295</v>
+      </c>
+      <c r="E4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" t="n">
         <v>395</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>390</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>-5</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>-60</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
@@ -660,23 +698,29 @@
         </is>
       </c>
       <c r="D5" t="n">
+        <v>228</v>
+      </c>
+      <c r="E5" t="n">
+        <v>82</v>
+      </c>
+      <c r="F5" t="n">
         <v>310</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>315</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>5</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>60</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>fuzzy</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
@@ -693,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -714,30 +758,40 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>wp_hausgeld</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>wp_ruecklage</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>wp_total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>actual_payment</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>delta_monthly</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>delta_annual</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>match_confidence</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
@@ -760,23 +814,29 @@
         </is>
       </c>
       <c r="D2" t="n">
+        <v>312</v>
+      </c>
+      <c r="E2" t="n">
+        <v>104</v>
+      </c>
+      <c r="F2" t="n">
         <v>416</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>420</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>4</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>48</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -799,23 +859,29 @@
         </is>
       </c>
       <c r="D3" t="n">
+        <v>308</v>
+      </c>
+      <c r="E3" t="n">
+        <v>105</v>
+      </c>
+      <c r="F3" t="n">
         <v>413</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>410</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>-3</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>-36</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -838,23 +904,29 @@
         </is>
       </c>
       <c r="D4" t="n">
+        <v>301</v>
+      </c>
+      <c r="E4" t="n">
+        <v>102</v>
+      </c>
+      <c r="F4" t="n">
         <v>403</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>400</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>-3</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>-36</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -877,23 +949,29 @@
         </is>
       </c>
       <c r="D5" t="n">
+        <v>245.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>89</v>
+      </c>
+      <c r="F5" t="n">
         <v>334.5</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>334.5</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -916,23 +994,29 @@
         </is>
       </c>
       <c r="D6" t="n">
+        <v>198</v>
+      </c>
+      <c r="E6" t="n">
+        <v>72</v>
+      </c>
+      <c r="F6" t="n">
         <v>270</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>270</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>0</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>fuzzy</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -955,23 +1039,29 @@
         </is>
       </c>
       <c r="D7" t="n">
+        <v>220</v>
+      </c>
+      <c r="E7" t="n">
+        <v>80</v>
+      </c>
+      <c r="F7" t="n">
         <v>300</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>300</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>0</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>0</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>fuzzy</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -994,23 +1084,29 @@
         </is>
       </c>
       <c r="D8" t="n">
+        <v>260</v>
+      </c>
+      <c r="E8" t="n">
+        <v>90</v>
+      </c>
+      <c r="F8" t="n">
         <v>350</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
         <v>350</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>fuzzy</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -1033,23 +1129,29 @@
         </is>
       </c>
       <c r="D9" t="n">
+        <v>215</v>
+      </c>
+      <c r="E9" t="n">
+        <v>78</v>
+      </c>
+      <c r="F9" t="n">
         <v>293</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
         <v>293</v>
       </c>
-      <c r="F9" t="n">
+      <c r="H9" t="n">
         <v>0</v>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>0</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -1072,23 +1174,29 @@
         </is>
       </c>
       <c r="D10" t="n">
+        <v>185</v>
+      </c>
+      <c r="E10" t="n">
+        <v>68</v>
+      </c>
+      <c r="F10" t="n">
         <v>253</v>
       </c>
-      <c r="E10" t="n">
+      <c r="G10" t="n">
         <v>253</v>
       </c>
-      <c r="F10" t="n">
+      <c r="H10" t="n">
         <v>0</v>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>fuzzy</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>

</xml_diff>